<commit_message>
Rio Grande do Sul no calendario; Sympla e Blueticket como fontes; roadrunners fora da pagina publica
- comum.UFS ganha RS: as fontes por estado rodam tambem para o RS; rs.html e a pagina do estado e todos.html vira Regiao Sul.
- Historico do RS: 2022 a 2025 do arquivo do corridasbr e concluintes do Open Results desde 2022.
- fontes.sympla (busca publica do site, pelo subtema de corrida) e fontes.blueticket (lista publica de eventos esportivos);
  o link do evento vira o link de inscricao (inscricao_url) e a data solta da ticketeira e acertada pela de outra fonte.
- build: FONTES_OCULTAS tira o roadrunners dos dados e dos cartoes da pagina publica (no BI continua).
- SEO, agendas, cadastro, parceiros e planilha modelo com o RS.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelo-calendario-provas.xlsx
+++ b/modelo-calendario-provas.xlsx
@@ -235,8 +235,8 @@
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="UF" error="Use SC ou PR." sqref="D2:D500">
-      <formula1>"SC,PR"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="UF" error="Use SC, PR ou RS." sqref="D2:D500">
+      <formula1>"SC,PR,RS"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Tipo" error="Escolha um tipo da lista." sqref="F2:F500">
       <formula1>"Rua,Trail,Caminhada,Kids,Revezamento,Noturna,Ultra,Duathlon,Triathlon,Outro"</formula1>
@@ -268,7 +268,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. Nome da prova, data, cidade e UF são obrigatórios. O calendário cobre SC e PR.</t>
+          <t xml:space="preserve">2. Nome da prova, data, cidade e UF são obrigatórios. O calendário cobre SC, PR e RS.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sao Paulo no calendario: 4.5 mil provas do corridasbr (2022-2026), Open Results, resultados pelo link e fotos; legenda dos numeros do cabecalho; laco do importar_ano corrigido
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelo-calendario-provas.xlsx
+++ b/modelo-calendario-provas.xlsx
@@ -235,8 +235,8 @@
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="UF" error="Use SC, PR ou RS." sqref="D2:D500">
-      <formula1>"SC,PR,RS"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="UF" error="Use SC, PR, RS ou SP." sqref="D2:D500">
+      <formula1>"SC,PR,RS,SP"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Tipo" error="Escolha um tipo da lista." sqref="F2:F500">
       <formula1>"Rua,Trail,Caminhada,Kids,Revezamento,Noturna,Ultra,Duathlon,Triathlon,Outro"</formula1>
@@ -268,7 +268,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. Nome da prova, data, cidade e UF são obrigatórios. O calendário cobre SC, PR e RS.</t>
+          <t xml:space="preserve">2. Nome da prova, data, cidade e UF são obrigatórios. O calendário cobre SC, PR, RS e SP.</t>
         </is>
       </c>
     </row>

</xml_diff>